<commit_message>
Add LADA natural history model and islet transplant outcomes analysis — Gap #1 and #3 GOLD computational dashboards
</commit_message>
<xml_diff>
--- a/Diabetes_Research_Tracker.xlsx
+++ b/Diabetes_Research_Tracker.xlsx
@@ -549,7 +549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K63"/>
+  <dimension ref="A1:K67"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="12" min="1" max="1"/>
@@ -3758,277 +3758,497 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
+      <c r="A59" s="12" t="inlineStr">
         <is>
           <t>T1D</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B59" s="12" t="inlineStr">
         <is>
           <t>Cure - Stem Cell</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C59" s="12" t="inlineStr">
         <is>
           <t>Autologous/Allogeneic Islet Therapy (Shi/Yin)</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr">
+      <c r="D59" s="12" t="inlineStr">
         <is>
           <t>Shanghai Changzheng Hospital</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
+      <c r="E59" s="12" t="inlineStr">
         <is>
           <t>iPSC-derived islets (autologous + allogeneic)</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr">
+      <c r="F59" s="12" t="inlineStr">
         <is>
           <t>Clinical Report</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr">
+      <c r="G59" s="12" t="inlineStr">
         <is>
           <t>Beta cell replacement</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr">
+      <c r="H59" s="12" t="inlineStr">
         <is>
           <t>3 T1D patients with complete beta cell loss; Lancet Diabetes Endocrinol 2026</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr">
+      <c r="I59" s="12" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="J59" t="n">
+      <c r="J59" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="K59" t="inlineStr">
+      <c r="K59" s="12" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/41765034/</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
+      <c r="A60" s="12" t="inlineStr">
         <is>
           <t>T2D</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="B60" s="12" t="inlineStr">
         <is>
           <t>Novel Mechanism</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C60" s="12" t="inlineStr">
         <is>
           <t>Canagliflozin Beta Cell Regeneration</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr">
+      <c r="D60" s="12" t="inlineStr">
         <is>
           <t>Popescu et al.</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr">
+      <c r="E60" s="12" t="inlineStr">
         <is>
           <t>SGLT2 inhibitor promoting beta cell regeneration &amp; identity</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr">
+      <c r="F60" s="12" t="inlineStr">
         <is>
           <t>Preclinical/Translational</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr">
+      <c r="G60" s="12" t="inlineStr">
         <is>
           <t>Beta cell recovery</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr">
+      <c r="H60" s="12" t="inlineStr">
         <is>
           <t>Promotes beta cell regeneration and restores beta cell identity in severe T2D model</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr">
+      <c r="I60" s="12" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="J60" t="n">
+      <c r="J60" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="K60" t="inlineStr">
+      <c r="K60" s="12" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/41814144/</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
+      <c r="A61" s="12" t="inlineStr">
         <is>
           <t>T2D</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
+      <c r="B61" s="12" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C61" s="12" t="inlineStr">
         <is>
           <t>MiniMed 780G for T2D</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr">
+      <c r="D61" s="12" t="inlineStr">
         <is>
           <t>Medtronic</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr">
+      <c r="E61" s="12" t="inlineStr">
         <is>
           <t>AID system with iAGC SmartGuard algorithm</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr">
+      <c r="F61" s="12" t="inlineStr">
         <is>
           <t>FDA Cleared</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr">
+      <c r="G61" s="12" t="inlineStr">
         <is>
           <t>Insulin-requiring T2D</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr">
+      <c r="H61" s="12" t="inlineStr">
         <is>
           <t>FDA cleared for T2D; Medicare access granted; ultra-rapid insulin cleared Feb 2026</t>
         </is>
       </c>
-      <c r="I61" t="inlineStr">
+      <c r="I61" s="12" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="J61" t="n">
+      <c r="J61" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="K61" t="inlineStr">
+      <c r="K61" s="12" t="inlineStr">
         <is>
           <t>https://news.medtronic.com/2026-02-02-Medtronic-Diabetes-expands-access</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
+      <c r="A62" s="12" t="inlineStr">
         <is>
           <t>T2D</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="B62" s="12" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C62" s="12" t="inlineStr">
         <is>
           <t>Dexcom G7 for Non-Insulin T2D</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr">
+      <c r="D62" s="12" t="inlineStr">
         <is>
           <t>Dexcom</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr">
+      <c r="E62" s="12" t="inlineStr">
         <is>
           <t>CGM for weight management and A1C in non-insulin T2D</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr">
+      <c r="F62" s="12" t="inlineStr">
         <is>
           <t>Registry Study</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr">
+      <c r="G62" s="12" t="inlineStr">
         <is>
           <t>Non-insulin T2D</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr">
+      <c r="H62" s="12" t="inlineStr">
         <is>
           <t>Long-term G7 use supports weight management and lowers A1C; ATTD 2026 data</t>
         </is>
       </c>
-      <c r="I62" t="inlineStr">
+      <c r="I62" s="12" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="J62" t="n">
+      <c r="J62" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="K62" t="inlineStr">
+      <c r="K62" s="12" t="inlineStr">
         <is>
           <t>https://investors.dexcom.com/news/news-details/2026/Dexcom-Showcases-Breakthrough-Outcomes</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
+      <c r="A63" s="12" t="inlineStr">
         <is>
           <t>T2D</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
+      <c r="B63" s="12" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="C63" s="12" t="inlineStr">
         <is>
           <t>Closed-Loop AID in T2D (Meta-Analysis)</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr">
+      <c r="D63" s="12" t="inlineStr">
         <is>
           <t>Ali et al.</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr">
+      <c r="E63" s="12" t="inlineStr">
         <is>
           <t>Systematic review of automated insulin delivery in T2D</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr">
+      <c r="F63" s="12" t="inlineStr">
         <is>
           <t>Meta-Analysis (1a)</t>
         </is>
       </c>
-      <c r="G63" t="inlineStr">
+      <c r="G63" s="12" t="inlineStr">
         <is>
           <t>T2D insulin users</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr">
+      <c r="H63" s="12" t="inlineStr">
         <is>
           <t>Meta-analysis of RCTs confirming AID efficacy in T2D</t>
         </is>
       </c>
-      <c r="I63" t="inlineStr">
+      <c r="I63" s="12" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="J63" t="n">
+      <c r="J63" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="K63" t="inlineStr">
+      <c r="K63" s="12" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/41830110/</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>T2D</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Oral GLP-1</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Ozempic Tablets (Oral Semaglutide)</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Novo Nordisk</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>GLP-1 receptor agonist (oral tablet formulation)</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>FDA Approved (Feb 2026)</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>T2D glycemic control</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>First oral GLP-1RA tablet; 25mg supplemental under review</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="J64" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>https://www.ajmc.com/view/fda-approves-oral-semaglutide-as-first-glp-1-pill-for-weight-loss</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>T2D</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Oral GLP-1</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>ASC30</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Ascletis Pharma</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Oral small molecule GLP-1 receptor agonist</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Phase 2 (IND cleared Mar 2026)</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>T2D</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>FDA IND cleared; enrollment starting Q1 2026</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Enrolling</t>
+        </is>
+      </c>
+      <c r="J65" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/ascletis-announces-us-fda-ind-clearance-for-13-week-phase-ii-study-of-its-oral-small-molecule-glp-1-asc30-in-participants-with-diabetes-302652107.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>T1D</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Cure - Immune Protection</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>MUSC Two-Part Cure (CAR-Treg + Stem Cell Islets)</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>MUSC / Breakthrough T1D</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Lab-made insulin-producing cells + engineered immune bodyguard cells</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Preclinical ($1M grant)</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>T1D functional cure without immunosuppression</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>$1M Breakthrough T1D grant (2026); two-part approach</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Preclinical</t>
+        </is>
+      </c>
+      <c r="J66" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>https://www.sciencedaily.com/releases/2026/03/260302030648.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>T1D</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Prevention</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Baricitinib (BARICADE Phase 3)</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Eli Lilly</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>JAK inhibitor for delay of Stage 3 T1D</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Phase 3 (NCT07222137)</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Delay Stage 3 T1D onset</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Phase 3 recruiting; JAK inhibitor preservation of beta cell function</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Recruiting</t>
+        </is>
+      </c>
+      <c r="J67" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>https://clinicaltrials.gov/study/NCT07222137</t>
         </is>
       </c>
     </row>
@@ -4922,7 +5142,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:K40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="35" customWidth="1" style="12" min="1" max="1"/>
@@ -6236,373 +6456,744 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="12" t="inlineStr">
         <is>
           <t>Autologous and allogeneic stem cell-derived islet therapy in three T1D recipients</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="12" t="inlineStr">
         <is>
           <t>Shi Y, Yin H et al.</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="12" t="inlineStr">
         <is>
           <t>Lancet Diabetes Endocrinol</t>
         </is>
       </c>
-      <c r="D27" t="n">
+      <c r="D27" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E27" s="12" t="inlineStr">
         <is>
           <t>T1D</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F27" s="12" t="inlineStr">
         <is>
           <t>Stem Cell Therapy</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G27" s="12" t="inlineStr">
         <is>
           <t>3 patients with complete beta cell loss received iPSC-derived islets; autologous + allogeneic approaches</t>
         </is>
       </c>
-      <c r="H27" t="n">
+      <c r="H27" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="I27" s="12" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="J27" s="12" t="inlineStr">
         <is>
           <t>BRONZE — single study, n=3. Triple-source: primary paper only; seek Lancet commentary + independent report</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="K27" s="12" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/S2213-8587(25)00423-1</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="12" t="inlineStr">
         <is>
           <t>Teplizumab Stage 2 T1D: Clinical Practice Experience (3 adults)</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="12" t="inlineStr">
         <is>
           <t>Guarnotta V et al.</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="12" t="inlineStr">
         <is>
           <t>Diabetes Obes Metab</t>
         </is>
       </c>
-      <c r="D28" t="n">
+      <c r="D28" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E28" s="12" t="inlineStr">
         <is>
           <t>T1D</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F28" s="12" t="inlineStr">
         <is>
           <t>Immunotherapy</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="G28" s="12" t="inlineStr">
         <is>
           <t>First Italian real-world teplizumab under compassionate use; feasible and safe in day-hospital setting</t>
         </is>
       </c>
-      <c r="H28" t="n">
+      <c r="H28" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="I28" s="12" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="J28" s="12" t="inlineStr">
         <is>
           <t>BRONZE — case series n=3. Cross-ref with Diabetologia real-world study (n=42) and Mahesh et al. DOM 2026</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
+      <c r="K28" s="12" t="inlineStr">
         <is>
           <t>https://doi.org/10.1111/dom.70626</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="12" t="inlineStr">
         <is>
           <t>Teplizumab real-world evaluation: metabolic and immunological outcomes</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="12" t="inlineStr">
         <is>
           <t>Karakus KE et al.</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="12" t="inlineStr">
         <is>
           <t>Diabetologia</t>
         </is>
       </c>
-      <c r="D29" t="n">
+      <c r="D29" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E29" s="12" t="inlineStr">
         <is>
           <t>T1D</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F29" s="12" t="inlineStr">
         <is>
           <t>Immunotherapy</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G29" s="12" t="inlineStr">
         <is>
           <t>First prospective real-world study post-FDA; n=30 treated vs n=10 control; 17% progressed at ~1yr</t>
         </is>
       </c>
-      <c r="H29" t="n">
+      <c r="H29" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="I29" s="12" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="J29" s="12" t="inlineStr">
         <is>
           <t>SILVER — prospective observational + consistent with RCT data</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
+      <c r="K29" s="12" t="inlineStr">
         <is>
           <t>https://doi.org/10.1007/s00125-025-06646-6</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="12" t="inlineStr">
         <is>
           <t>Canagliflozin promotes beta-cell regeneration and restores beta-cell identity</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="12" t="inlineStr">
         <is>
           <t>Popescu I et al.</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="12" t="inlineStr">
         <is>
           <t>J Cell Mol Med</t>
         </is>
       </c>
-      <c r="D30" t="n">
+      <c r="D30" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E30" s="12" t="inlineStr">
         <is>
           <t>T2D</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="F30" s="12" t="inlineStr">
         <is>
           <t>Beta Cell / SGLT2i</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="G30" s="12" t="inlineStr">
         <is>
           <t>SGLT2 inhibitor promotes beta cell regeneration and restores beta cell identity in polygenic T2D model</t>
         </is>
       </c>
-      <c r="H30" t="n">
+      <c r="H30" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="I30" s="12" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="J30" s="12" t="inlineStr">
         <is>
           <t>BRONZE — preclinical (animal model). Prior: dapagliflozin similar (PMID:32712220). Drug repurposing relevance.</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr">
+      <c r="K30" s="12" t="inlineStr">
         <is>
           <t>https://doi.org/10.1111/jcmm.71041</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="12" t="inlineStr">
         <is>
           <t>Closed-Loop AID in T2D: Meta-Analysis of RCTs</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="12" t="inlineStr">
         <is>
           <t>Ali D et al.</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="12" t="inlineStr">
         <is>
           <t>Endocrinol Diabetes Metab</t>
         </is>
       </c>
-      <c r="D31" t="n">
+      <c r="D31" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E31" s="12" t="inlineStr">
         <is>
           <t>T2D</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F31" s="12" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G31" s="12" t="inlineStr">
         <is>
           <t>Systematic review/meta-analysis of RCTs confirming AID efficacy for insulin-requiring T2D patients</t>
         </is>
       </c>
-      <c r="H31" t="n">
+      <c r="H31" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="I31" s="12" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="J31" s="12" t="inlineStr">
         <is>
           <t>Evidence Level 1a. Supports expanding AID beyond T1D.</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
+      <c r="K31" s="12" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/edm2.70178</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="12" t="inlineStr">
         <is>
           <t>EASD/ADA Position: Individualizing Diabetes Technology</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="12" t="inlineStr">
         <is>
           <t>Bruttomesso D et al.</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="12" t="inlineStr">
         <is>
           <t>Diabetes Care + Diabetologia</t>
         </is>
       </c>
-      <c r="D32" t="n">
+      <c r="D32" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E32" s="12" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F32" s="12" t="inlineStr">
         <is>
           <t>Technology / Equity</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G32" s="12" t="inlineStr">
         <is>
           <t>Joint position: individualized tech approach; CGM at diagnosis; fewer restrictions on AID initiation</t>
         </is>
       </c>
-      <c r="H32" t="n">
+      <c r="H32" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="I32" s="12" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="J32" s="12" t="inlineStr">
         <is>
           <t>Evidence Level G (guideline). Dual-published EASD+ADA. Impacts all technology access analysis.</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="K32" s="12" t="inlineStr">
         <is>
           <t>https://doi.org/10.2337/dci26-0018</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="12" t="inlineStr">
         <is>
           <t>Orforglipron superior to oral semaglutide: ACHIEVE-3 results</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="12" t="inlineStr">
         <is>
           <t>Eli Lilly / Multiple</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="12" t="inlineStr">
         <is>
           <t>The Lancet</t>
         </is>
       </c>
-      <c r="D33" t="n">
+      <c r="D33" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E33" s="12" t="inlineStr">
         <is>
           <t>T2D</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F33" s="12" t="inlineStr">
         <is>
           <t>GLP-1 Oral</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="G33" s="12" t="inlineStr">
         <is>
           <t>Head-to-head Phase 3: orforglipron superior glycemic control vs oral semaglutide in T2D</t>
         </is>
       </c>
-      <c r="H33" t="n">
+      <c r="H33" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="I33" s="12" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="J33" s="12" t="inlineStr">
         <is>
           <t>SILVER — Phase 3 RCT, peer-reviewed; FDA action date Apr 10 2026</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr">
+      <c r="K33" s="12" t="inlineStr">
         <is>
           <t>https://investor.lilly.com/news-releases/news-release-details/lillys-oral-glp-1-orforglipron-delivered-superior-blood-sugar</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Teplizumab Stage 2 T1D: Clinical Practice Experience (3 adults)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Guarnotta V et al.</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Diabetes Obes Metab</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>T1D</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Immunotherapy/Prevention</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Real-world data on Tzield in 3 adult Stage 2 patients</t>
+        </is>
+      </c>
+      <c r="H34" t="n">
+        <v>4</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>KEY THERAPY — first clinical practice report for teplizumab</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/dom.70626</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Use of CGM to stratify individuals without diabetes</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Communications Medicine authors</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Communications Medicine</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>AI/ML</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Technology/Prediction</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>CGM data for pre-diabetes risk stratification</t>
+        </is>
+      </c>
+      <c r="H35" t="n">
+        <v>4</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Tier 1 relevance: AI/ML Prediction Model Development</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/41832215/</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>High-Fidelity Synthetic Data Replicates Clinical Prediction in Million-Patient Diabetes Cohort</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Ortuño F et al.</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Advanced Science</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>AI/ML</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Methodology</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Synthetic data replicates clinical prediction performance</t>
+        </is>
+      </c>
+      <c r="H36" t="n">
+        <v>4</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Methodological advance for data-limited settings</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/advs.202516196</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Semaglutide as add-on therapy in LADA</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Lunati ME et al.</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>J Clin Endocrinol Metab</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LADA</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Treatment</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Semaglutide adjunctive therapy in LADA patients</t>
+        </is>
+      </c>
+      <c r="H37" t="n">
+        <v>5</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>HIGH PRIORITY — LADA is most neglected subtype; novel treatment approach</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1210/clinem/dgag072</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>SGLT2 Inhibitor Canagliflozin Promotes β-Cell Regeneration in T2D</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Popescu I et al.</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>J Cell Mol Med</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>T2D</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Beta Cell Regen</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Canagliflozin promotes beta-cell regeneration and restores identity in polygenic T2D model</t>
+        </is>
+      </c>
+      <c r="H38" t="n">
+        <v>4</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Drug repurposing angle — existing drug with novel regenerative mechanism</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/jcmm.71041</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Polysaccharide [triple-domain cross-domain paper]</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Zhu R et al.</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>J Agric Food Chem</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Biomarker/Microbiome/Complications</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Cross-Domain</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Spans Biomarker + Microbiome + Complications domains</t>
+        </is>
+      </c>
+      <c r="H39" t="n">
+        <v>3</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>CROSS-DOMAIN: Triple-domain paper — highest synthesis value</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1021/acs.jafc.5c16173</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>XAI methods for clinically meaningful glycemia prediction explanations</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Rotbei S et al.</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>BMC Med Inform Decis Mak</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>AI/ML</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Explainability</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Explainable AI for diabetes glycemia prediction</t>
+        </is>
+      </c>
+      <c r="H40" t="n">
+        <v>3</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Relevant to responsible AI in clinical diabetes prediction</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1186/s12911-026-03420-5</t>
         </is>
       </c>
     </row>
@@ -7797,7 +8388,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="35" customWidth="1" style="12" min="1" max="1"/>
@@ -7991,35 +8582,67 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>Last Updated</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>2026-03-15</t>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>Active FDA Reviews (2026)</t>
         </is>
       </c>
-      <c r="B19" t="n">
-        <v>3</v>
+      <c r="B19" s="12" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="12" t="inlineStr">
         <is>
           <t>Phase 3 Recruiting (from API)</t>
         </is>
       </c>
-      <c r="B20" t="n">
+      <c r="B20" s="12" t="n">
         <v>42</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Cross-Domain Papers (Current)</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>PubMed Unique Papers (30-day)</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Monitor Report Date</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily iteration Run 24: Vet PMID 40907678, add 2 new papers (41546551, 41020547), Monday search, pipeline rebuild all 39 OK
</commit_message>
<xml_diff>
--- a/Diabetes_Research_Tracker.xlsx
+++ b/Diabetes_Research_Tracker.xlsx
@@ -26,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -77,6 +77,10 @@
       <family val="0"/>
       <b val="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="8">
@@ -157,7 +161,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -230,6 +234,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -549,7 +556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K67"/>
+  <dimension ref="A1:K73"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="12" min="1" max="1"/>
@@ -4033,222 +4040,552 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
+      <c r="A64" s="12" t="inlineStr">
         <is>
           <t>T2D</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B64" s="12" t="inlineStr">
         <is>
           <t>Oral GLP-1</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C64" s="12" t="inlineStr">
         <is>
           <t>Ozempic Tablets (Oral Semaglutide)</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr">
+      <c r="D64" s="12" t="inlineStr">
         <is>
           <t>Novo Nordisk</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr">
+      <c r="E64" s="12" t="inlineStr">
         <is>
           <t>GLP-1 receptor agonist (oral tablet formulation)</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr">
+      <c r="F64" s="12" t="inlineStr">
         <is>
           <t>FDA Approved (Feb 2026)</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr">
+      <c r="G64" s="12" t="inlineStr">
         <is>
           <t>T2D glycemic control</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr">
+      <c r="H64" s="12" t="inlineStr">
         <is>
           <t>First oral GLP-1RA tablet; 25mg supplemental under review</t>
         </is>
       </c>
-      <c r="I64" t="inlineStr">
+      <c r="I64" s="12" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="J64" t="n">
+      <c r="J64" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="K64" t="inlineStr">
+      <c r="K64" s="12" t="inlineStr">
         <is>
           <t>https://www.ajmc.com/view/fda-approves-oral-semaglutide-as-first-glp-1-pill-for-weight-loss</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
+      <c r="A65" s="12" t="inlineStr">
         <is>
           <t>T2D</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
+      <c r="B65" s="12" t="inlineStr">
         <is>
           <t>Oral GLP-1</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="C65" s="12" t="inlineStr">
         <is>
           <t>ASC30</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr">
+      <c r="D65" s="12" t="inlineStr">
         <is>
           <t>Ascletis Pharma</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
+      <c r="E65" s="12" t="inlineStr">
         <is>
           <t>Oral small molecule GLP-1 receptor agonist</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr">
+      <c r="F65" s="12" t="inlineStr">
         <is>
           <t>Phase 2 (IND cleared Mar 2026)</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr">
+      <c r="G65" s="12" t="inlineStr">
         <is>
           <t>T2D</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr">
+      <c r="H65" s="12" t="inlineStr">
         <is>
           <t>FDA IND cleared; enrollment starting Q1 2026</t>
         </is>
       </c>
-      <c r="I65" t="inlineStr">
+      <c r="I65" s="12" t="inlineStr">
         <is>
           <t>Enrolling</t>
         </is>
       </c>
-      <c r="J65" t="n">
+      <c r="J65" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="K65" t="inlineStr">
+      <c r="K65" s="12" t="inlineStr">
         <is>
           <t>https://www.prnewswire.com/news-releases/ascletis-announces-us-fda-ind-clearance-for-13-week-phase-ii-study-of-its-oral-small-molecule-glp-1-asc30-in-participants-with-diabetes-302652107.html</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
+      <c r="A66" s="12" t="inlineStr">
         <is>
           <t>T1D</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="B66" s="12" t="inlineStr">
         <is>
           <t>Cure - Immune Protection</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C66" s="12" t="inlineStr">
         <is>
           <t>MUSC Two-Part Cure (CAR-Treg + Stem Cell Islets)</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr">
+      <c r="D66" s="12" t="inlineStr">
         <is>
           <t>MUSC / Breakthrough T1D</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr">
+      <c r="E66" s="12" t="inlineStr">
         <is>
           <t>Lab-made insulin-producing cells + engineered immune bodyguard cells</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr">
+      <c r="F66" s="12" t="inlineStr">
         <is>
           <t>Preclinical ($1M grant)</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr">
+      <c r="G66" s="12" t="inlineStr">
         <is>
           <t>T1D functional cure without immunosuppression</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr">
+      <c r="H66" s="12" t="inlineStr">
         <is>
           <t>$1M Breakthrough T1D grant (2026); two-part approach</t>
         </is>
       </c>
-      <c r="I66" t="inlineStr">
+      <c r="I66" s="12" t="inlineStr">
         <is>
           <t>Preclinical</t>
         </is>
       </c>
-      <c r="J66" t="n">
+      <c r="J66" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="K66" t="inlineStr">
+      <c r="K66" s="12" t="inlineStr">
         <is>
           <t>https://www.sciencedaily.com/releases/2026/03/260302030648.htm</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
+      <c r="A67" s="12" t="inlineStr">
         <is>
           <t>T1D</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr">
+      <c r="B67" s="12" t="inlineStr">
         <is>
           <t>Prevention</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr">
+      <c r="C67" s="12" t="inlineStr">
         <is>
           <t>Baricitinib (BARICADE Phase 3)</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr">
+      <c r="D67" s="12" t="inlineStr">
         <is>
           <t>Eli Lilly</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr">
+      <c r="E67" s="12" t="inlineStr">
         <is>
           <t>JAK inhibitor for delay of Stage 3 T1D</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr">
+      <c r="F67" s="12" t="inlineStr">
         <is>
           <t>Phase 3 (NCT07222137)</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr">
+      <c r="G67" s="12" t="inlineStr">
         <is>
           <t>Delay Stage 3 T1D onset</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr">
+      <c r="H67" s="12" t="inlineStr">
         <is>
           <t>Phase 3 recruiting; JAK inhibitor preservation of beta cell function</t>
         </is>
       </c>
-      <c r="I67" t="inlineStr">
+      <c r="I67" s="12" t="inlineStr">
         <is>
           <t>Recruiting</t>
         </is>
       </c>
-      <c r="J67" t="n">
+      <c r="J67" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="K67" t="inlineStr">
+      <c r="K67" s="12" t="inlineStr">
         <is>
           <t>https://clinicaltrials.gov/study/NCT07222137</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="25" t="inlineStr">
+        <is>
+          <t>T1D</t>
+        </is>
+      </c>
+      <c r="B68" s="25" t="inlineStr">
+        <is>
+          <t>Immunotherapy</t>
+        </is>
+      </c>
+      <c r="C68" s="25" t="inlineStr">
+        <is>
+          <t>Rezpegaldesleukin (NKTR-358)</t>
+        </is>
+      </c>
+      <c r="D68" s="25" t="inlineStr">
+        <is>
+          <t>Nektar Therapeutics</t>
+        </is>
+      </c>
+      <c r="E68" s="25" t="inlineStr">
+        <is>
+          <t>IL-2 conjugate for selective Treg expansion</t>
+        </is>
+      </c>
+      <c r="F68" s="25" t="inlineStr">
+        <is>
+          <t>Phase (TBD) (NCT07142252)</t>
+        </is>
+      </c>
+      <c r="G68" s="25" t="inlineStr">
+        <is>
+          <t>New Onset T1D</t>
+        </is>
+      </c>
+      <c r="H68" s="25" t="inlineStr">
+        <is>
+          <t>IL-2 pathway Treg expansion; began recruiting April 2026</t>
+        </is>
+      </c>
+      <c r="I68" s="25" t="inlineStr">
+        <is>
+          <t>Recruiting</t>
+        </is>
+      </c>
+      <c r="J68" s="25" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K68" s="25" t="inlineStr">
+        <is>
+          <t>https://clinicaltrials.gov/study/NCT07142252</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="25" t="inlineStr">
+        <is>
+          <t>T2D</t>
+        </is>
+      </c>
+      <c r="B69" s="25" t="inlineStr">
+        <is>
+          <t>Oral GLP-1</t>
+        </is>
+      </c>
+      <c r="C69" s="25" t="inlineStr">
+        <is>
+          <t>Foundayo (Orforglipron)</t>
+        </is>
+      </c>
+      <c r="D69" s="25" t="inlineStr">
+        <is>
+          <t>Eli Lilly</t>
+        </is>
+      </c>
+      <c r="E69" s="25" t="inlineStr">
+        <is>
+          <t>Oral non-peptide GLP-1 receptor agonist</t>
+        </is>
+      </c>
+      <c r="F69" s="25" t="inlineStr">
+        <is>
+          <t>FDA Approved (Apr 1, 2026)</t>
+        </is>
+      </c>
+      <c r="G69" s="25" t="inlineStr">
+        <is>
+          <t>Obesity/overweight (T2D indication pending)</t>
+        </is>
+      </c>
+      <c r="H69" s="25" t="inlineStr">
+        <is>
+          <t>First oral non-peptide GLP-1 pill; approved under CNPV program 294 days ahead of PDUFA; any time of day dosing without food/water restrictions</t>
+        </is>
+      </c>
+      <c r="I69" s="25" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="J69" s="25" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K69" s="25" t="inlineStr">
+        <is>
+          <t>https://www.hcplive.com/view/diabetes-dialogue-orforglipron-receives-fda-approval-for-chronic-weight-management</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="25" t="inlineStr">
+        <is>
+          <t>T2D</t>
+        </is>
+      </c>
+      <c r="B70" s="25" t="inlineStr">
+        <is>
+          <t>Biosimilar</t>
+        </is>
+      </c>
+      <c r="C70" s="25" t="inlineStr">
+        <is>
+          <t>Merilog (Biosimilar Insulin Aspart)</t>
+        </is>
+      </c>
+      <c r="D70" s="25" t="inlineStr">
+        <is>
+          <t>FDA-approved biosimilar</t>
+        </is>
+      </c>
+      <c r="E70" s="25" t="inlineStr">
+        <is>
+          <t>Biosimilar of insulin aspart (Novolog)</t>
+        </is>
+      </c>
+      <c r="F70" s="25" t="inlineStr">
+        <is>
+          <t>FDA Approved (Mar 2026)</t>
+        </is>
+      </c>
+      <c r="G70" s="25" t="inlineStr">
+        <is>
+          <t>Diabetes (T1D/T2D)</t>
+        </is>
+      </c>
+      <c r="H70" s="25" t="inlineStr">
+        <is>
+          <t>Biosimilar insulin aspart; expands insulin access options</t>
+        </is>
+      </c>
+      <c r="I70" s="25" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="J70" s="25" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K70" s="25" t="inlineStr">
+        <is>
+          <t>https://www.hcplive.com/view/fda-approves-merilog-biosimilar-product-insulin-aspart-novolog-diabetes</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="25" t="inlineStr">
+        <is>
+          <t>T2D</t>
+        </is>
+      </c>
+      <c r="B71" s="25" t="inlineStr">
+        <is>
+          <t>Novel Insulin</t>
+        </is>
+      </c>
+      <c r="C71" s="25" t="inlineStr">
+        <is>
+          <t>Awiqli (Insulin Icodec)</t>
+        </is>
+      </c>
+      <c r="D71" s="25" t="inlineStr">
+        <is>
+          <t>Novo Nordisk</t>
+        </is>
+      </c>
+      <c r="E71" s="25" t="inlineStr">
+        <is>
+          <t>Once-weekly basal insulin</t>
+        </is>
+      </c>
+      <c r="F71" s="25" t="inlineStr">
+        <is>
+          <t>FDA Approved (Mar 27, 2026)</t>
+        </is>
+      </c>
+      <c r="G71" s="25" t="inlineStr">
+        <is>
+          <t>T2D glycemic control</t>
+        </is>
+      </c>
+      <c r="H71" s="25" t="inlineStr">
+        <is>
+          <t>First once-weekly basal insulin; reduces injections from 7 to 1 per week; nationwide availability H2 2026</t>
+        </is>
+      </c>
+      <c r="I71" s="25" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="J71" s="25" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K71" s="25" t="inlineStr">
+        <is>
+          <t>https://www.roi-nj.com/2026/04/02/healthcare/fda-approves-novo-nordisks-awiqli-a-once-weekly-basal-insulin-treatment-for-adults-with-type-2-diabetes/</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="25" t="inlineStr">
+        <is>
+          <t>T2D</t>
+        </is>
+      </c>
+      <c r="B72" s="25" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C72" s="25" t="inlineStr">
+        <is>
+          <t>MiniMed Flex AID System</t>
+        </is>
+      </c>
+      <c r="D72" s="25" t="inlineStr">
+        <is>
+          <t>Medtronic</t>
+        </is>
+      </c>
+      <c r="E72" s="25" t="inlineStr">
+        <is>
+          <t>Automated insulin delivery system</t>
+        </is>
+      </c>
+      <c r="F72" s="25" t="inlineStr">
+        <is>
+          <t>FDA Cleared (Mar 18, 2026)</t>
+        </is>
+      </c>
+      <c r="G72" s="25" t="inlineStr">
+        <is>
+          <t>T1D (≥7yr) and insulin-requiring T2D</t>
+        </is>
+      </c>
+      <c r="H72" s="25" t="inlineStr">
+        <is>
+          <t>New AID system cleared for ages ≥7 with T1D and adults with insulin-requiring T2D</t>
+        </is>
+      </c>
+      <c r="I72" s="25" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="J72" s="25" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K72" s="25" t="inlineStr">
+        <is>
+          <t>https://news.medtronic.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="25" t="inlineStr">
+        <is>
+          <t>T2D</t>
+        </is>
+      </c>
+      <c r="B73" s="25" t="inlineStr">
+        <is>
+          <t>Novel Mechanism</t>
+        </is>
+      </c>
+      <c r="C73" s="25" t="inlineStr">
+        <is>
+          <t>Icovamenib (Biomea Fusion)</t>
+        </is>
+      </c>
+      <c r="D73" s="25" t="inlineStr">
+        <is>
+          <t>Biomea Fusion</t>
+        </is>
+      </c>
+      <c r="E73" s="25" t="inlineStr">
+        <is>
+          <t>Menin inhibitor for beta cell regeneration</t>
+        </is>
+      </c>
+      <c r="F73" s="25" t="inlineStr">
+        <is>
+          <t>Phase 2 (NCT07502495, NCT07502508)</t>
+        </is>
+      </c>
+      <c r="G73" s="25" t="inlineStr">
+        <is>
+          <t>T2D beta cell restoration</t>
+        </is>
+      </c>
+      <c r="H73" s="25" t="inlineStr">
+        <is>
+          <t>Novel menin inhibitor; Phase 2 expansion initiated April 2026</t>
+        </is>
+      </c>
+      <c r="I73" s="25" t="inlineStr">
+        <is>
+          <t>Recruiting</t>
+        </is>
+      </c>
+      <c r="J73" s="25" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K73" s="25" t="inlineStr">
+        <is>
+          <t>https://clinicaltrials.gov/study/NCT07502495</t>
         </is>
       </c>
     </row>
@@ -6827,371 +7164,371 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="12" t="inlineStr">
         <is>
           <t>Teplizumab Stage 2 T1D: Clinical Practice Experience (3 adults)</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="12" t="inlineStr">
         <is>
           <t>Guarnotta V et al.</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="12" t="inlineStr">
         <is>
           <t>Diabetes Obes Metab</t>
         </is>
       </c>
-      <c r="D34" t="n">
+      <c r="D34" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E34" s="12" t="inlineStr">
         <is>
           <t>T1D</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F34" s="12" t="inlineStr">
         <is>
           <t>Immunotherapy/Prevention</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="G34" s="12" t="inlineStr">
         <is>
           <t>Real-world data on Tzield in 3 adult Stage 2 patients</t>
         </is>
       </c>
-      <c r="H34" t="n">
+      <c r="H34" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="I34" s="12" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="J34" s="12" t="inlineStr">
         <is>
           <t>KEY THERAPY — first clinical practice report for teplizumab</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr">
+      <c r="K34" s="12" t="inlineStr">
         <is>
           <t>https://doi.org/10.1111/dom.70626</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="12" t="inlineStr">
         <is>
           <t>Use of CGM to stratify individuals without diabetes</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="12" t="inlineStr">
         <is>
           <t>Communications Medicine authors</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="12" t="inlineStr">
         <is>
           <t>Communications Medicine</t>
         </is>
       </c>
-      <c r="D35" t="n">
+      <c r="D35" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E35" s="12" t="inlineStr">
         <is>
           <t>AI/ML</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F35" s="12" t="inlineStr">
         <is>
           <t>Technology/Prediction</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="G35" s="12" t="inlineStr">
         <is>
           <t>CGM data for pre-diabetes risk stratification</t>
         </is>
       </c>
-      <c r="H35" t="n">
+      <c r="H35" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="I35" s="12" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr">
+      <c r="J35" s="12" t="inlineStr">
         <is>
           <t>Tier 1 relevance: AI/ML Prediction Model Development</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr">
+      <c r="K35" s="12" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/41832215/</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="12" t="inlineStr">
         <is>
           <t>High-Fidelity Synthetic Data Replicates Clinical Prediction in Million-Patient Diabetes Cohort</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="12" t="inlineStr">
         <is>
           <t>Ortuño F et al.</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="12" t="inlineStr">
         <is>
           <t>Advanced Science</t>
         </is>
       </c>
-      <c r="D36" t="n">
+      <c r="D36" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E36" s="12" t="inlineStr">
         <is>
           <t>AI/ML</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F36" s="12" t="inlineStr">
         <is>
           <t>Methodology</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="G36" s="12" t="inlineStr">
         <is>
           <t>Synthetic data replicates clinical prediction performance</t>
         </is>
       </c>
-      <c r="H36" t="n">
+      <c r="H36" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="I36" t="inlineStr">
+      <c r="I36" s="12" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr">
+      <c r="J36" s="12" t="inlineStr">
         <is>
           <t>Methodological advance for data-limited settings</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr">
+      <c r="K36" s="12" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/advs.202516196</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="12" t="inlineStr">
         <is>
           <t>Semaglutide as add-on therapy in LADA</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="12" t="inlineStr">
         <is>
           <t>Lunati ME et al.</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="12" t="inlineStr">
         <is>
           <t>J Clin Endocrinol Metab</t>
         </is>
       </c>
-      <c r="D37" t="n">
+      <c r="D37" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E37" s="12" t="inlineStr">
         <is>
           <t>LADA</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F37" s="12" t="inlineStr">
         <is>
           <t>Treatment</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="G37" s="12" t="inlineStr">
         <is>
           <t>Semaglutide adjunctive therapy in LADA patients</t>
         </is>
       </c>
-      <c r="H37" t="n">
+      <c r="H37" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="I37" t="inlineStr">
+      <c r="I37" s="12" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr">
+      <c r="J37" s="12" t="inlineStr">
         <is>
           <t>HIGH PRIORITY — LADA is most neglected subtype; novel treatment approach</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr">
+      <c r="K37" s="12" t="inlineStr">
         <is>
           <t>https://doi.org/10.1210/clinem/dgag072</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="12" t="inlineStr">
         <is>
           <t>SGLT2 Inhibitor Canagliflozin Promotes β-Cell Regeneration in T2D</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="12" t="inlineStr">
         <is>
           <t>Popescu I et al.</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="12" t="inlineStr">
         <is>
           <t>J Cell Mol Med</t>
         </is>
       </c>
-      <c r="D38" t="n">
+      <c r="D38" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E38" s="12" t="inlineStr">
         <is>
           <t>T2D</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F38" s="12" t="inlineStr">
         <is>
           <t>Beta Cell Regen</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="G38" s="12" t="inlineStr">
         <is>
           <t>Canagliflozin promotes beta-cell regeneration and restores identity in polygenic T2D model</t>
         </is>
       </c>
-      <c r="H38" t="n">
+      <c r="H38" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="I38" s="12" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr">
+      <c r="J38" s="12" t="inlineStr">
         <is>
           <t>Drug repurposing angle — existing drug with novel regenerative mechanism</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr">
+      <c r="K38" s="12" t="inlineStr">
         <is>
           <t>https://doi.org/10.1111/jcmm.71041</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="12" t="inlineStr">
         <is>
           <t>Polysaccharide [triple-domain cross-domain paper]</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="12" t="inlineStr">
         <is>
           <t>Zhu R et al.</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="12" t="inlineStr">
         <is>
           <t>J Agric Food Chem</t>
         </is>
       </c>
-      <c r="D39" t="n">
+      <c r="D39" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E39" s="12" t="inlineStr">
         <is>
           <t>Biomarker/Microbiome/Complications</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F39" s="12" t="inlineStr">
         <is>
           <t>Cross-Domain</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="G39" s="12" t="inlineStr">
         <is>
           <t>Spans Biomarker + Microbiome + Complications domains</t>
         </is>
       </c>
-      <c r="H39" t="n">
+      <c r="H39" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="I39" s="12" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr">
+      <c r="J39" s="12" t="inlineStr">
         <is>
           <t>CROSS-DOMAIN: Triple-domain paper — highest synthesis value</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
+      <c r="K39" s="12" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/acs.jafc.5c16173</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="12" t="inlineStr">
         <is>
           <t>XAI methods for clinically meaningful glycemia prediction explanations</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="12" t="inlineStr">
         <is>
           <t>Rotbei S et al.</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="12" t="inlineStr">
         <is>
           <t>BMC Med Inform Decis Mak</t>
         </is>
       </c>
-      <c r="D40" t="n">
+      <c r="D40" s="12" t="n">
         <v>2026</v>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E40" s="12" t="inlineStr">
         <is>
           <t>AI/ML</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F40" s="12" t="inlineStr">
         <is>
           <t>Explainability</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
+      <c r="G40" s="12" t="inlineStr">
         <is>
           <t>Explainable AI for diabetes glycemia prediction</t>
         </is>
       </c>
-      <c r="H40" t="n">
+      <c r="H40" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="I40" t="inlineStr">
+      <c r="I40" s="12" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr">
+      <c r="J40" s="12" t="inlineStr">
         <is>
           <t>Relevant to responsible AI in clinical diabetes prediction</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr">
+      <c r="K40" s="12" t="inlineStr">
         <is>
           <t>https://doi.org/10.1186/s12911-026-03420-5</t>
         </is>
@@ -8413,8 +8750,9 @@
           <t>Total Pipeline Entries</t>
         </is>
       </c>
-      <c r="B2" s="24" t="n">
-        <v>62</v>
+      <c r="B2" s="24">
+        <f>COUNTA('Therapy Pipeline'!A2:A74)</f>
+        <v/>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="13">
@@ -8589,7 +8927,7 @@
       </c>
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-04-03</t>
         </is>
       </c>
     </row>
@@ -8600,7 +8938,7 @@
         </is>
       </c>
       <c r="B19" s="12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20">
@@ -8610,38 +8948,38 @@
         </is>
       </c>
       <c r="B20" s="12" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="12" t="inlineStr">
         <is>
           <t>Cross-Domain Papers (Current)</t>
         </is>
       </c>
-      <c r="B21" t="n">
-        <v>10</v>
+      <c r="B21" s="12" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="12" t="inlineStr">
         <is>
           <t>PubMed Unique Papers (30-day)</t>
         </is>
       </c>
-      <c r="B22" t="n">
-        <v>124</v>
+      <c r="B22" s="12" t="n">
+        <v>129</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="12" t="inlineStr">
         <is>
           <t>Monitor Report Date</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>2026-03-16</t>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily iteration: vetted 15 papers, validated 3 paths (metformin/HCQ/NLRP3), pipeline OK
</commit_message>
<xml_diff>
--- a/Diabetes_Research_Tracker.xlsx
+++ b/Diabetes_Research_Tracker.xlsx
@@ -83,7 +83,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -126,6 +126,11 @@
         <bgColor rgb="FF7B2D8E"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFCC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -161,7 +166,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -238,6 +243,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -556,7 +562,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K73"/>
+  <dimension ref="A1:K77"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="12" min="1" max="1"/>
@@ -4586,6 +4592,226 @@
       <c r="K73" s="25" t="inlineStr">
         <is>
           <t>https://clinicaltrials.gov/study/NCT07502495</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="26" t="inlineStr">
+        <is>
+          <t>T2D</t>
+        </is>
+      </c>
+      <c r="B74" s="26" t="inlineStr">
+        <is>
+          <t>Insulin - Weekly Basal</t>
+        </is>
+      </c>
+      <c r="C74" s="26" t="inlineStr">
+        <is>
+          <t>Awiqli (insulin icodec)</t>
+        </is>
+      </c>
+      <c r="D74" s="26" t="inlineStr">
+        <is>
+          <t>Novo Nordisk</t>
+        </is>
+      </c>
+      <c r="E74" s="26" t="inlineStr">
+        <is>
+          <t>Once-weekly basal insulin</t>
+        </is>
+      </c>
+      <c r="F74" s="26" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="G74" s="26" t="inlineStr">
+        <is>
+          <t>Reduce injection burden</t>
+        </is>
+      </c>
+      <c r="H74" s="26" t="inlineStr">
+        <is>
+          <t>FDA approved March 2026 — first once-weekly basal insulin for T2D. Phase 3 trial NCT07076199 testing in T1D.</t>
+        </is>
+      </c>
+      <c r="I74" s="26" t="inlineStr">
+        <is>
+          <t>FDA Approved (T2D)</t>
+        </is>
+      </c>
+      <c r="J74" s="26" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K74" s="26" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/fda-approves-novo-nordisks-awiqli-the-first-and-only-once-weekly-basal-insulin-treatment-for-adults-with-type-2-diabetes-302726839.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="26" t="inlineStr">
+        <is>
+          <t>T2D</t>
+        </is>
+      </c>
+      <c r="B75" s="26" t="inlineStr">
+        <is>
+          <t>SGLT2i - Generic Access</t>
+        </is>
+      </c>
+      <c r="C75" s="26" t="inlineStr">
+        <is>
+          <t>Generic Dapagliflozin (Farxiga)</t>
+        </is>
+      </c>
+      <c r="D75" s="26" t="inlineStr">
+        <is>
+          <t>Multiple (FDA generic approval)</t>
+        </is>
+      </c>
+      <c r="E75" s="26" t="inlineStr">
+        <is>
+          <t>SGLT2 inhibition</t>
+        </is>
+      </c>
+      <c r="F75" s="26" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="G75" s="26" t="inlineStr">
+        <is>
+          <t>Broaden SGLT2i access</t>
+        </is>
+      </c>
+      <c r="H75" s="26" t="inlineStr">
+        <is>
+          <t>First generics of Farxiga approved April 2026 for HF risk reduction in T2D + glycemic control. Increases access.</t>
+        </is>
+      </c>
+      <c r="I75" s="26" t="inlineStr">
+        <is>
+          <t>FDA Approved (Generic)</t>
+        </is>
+      </c>
+      <c r="J75" s="26" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K75" s="26" t="inlineStr">
+        <is>
+          <t>https://www.fda.gov/drugs/drug-alerts-and-statements/fda-approves-first-generic-dapagliflozin-tablets</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="26" t="inlineStr">
+        <is>
+          <t>T2D</t>
+        </is>
+      </c>
+      <c r="B76" s="26" t="inlineStr">
+        <is>
+          <t>SGLT2i + Metformin - Generic</t>
+        </is>
+      </c>
+      <c r="C76" s="26" t="inlineStr">
+        <is>
+          <t>Generic Dapagliflozin-Metformin</t>
+        </is>
+      </c>
+      <c r="D76" s="26" t="inlineStr">
+        <is>
+          <t>Lupin</t>
+        </is>
+      </c>
+      <c r="E76" s="26" t="inlineStr">
+        <is>
+          <t>SGLT2i + biguanide combo</t>
+        </is>
+      </c>
+      <c r="F76" s="26" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="G76" s="26" t="inlineStr">
+        <is>
+          <t>Lower-cost T2D combo</t>
+        </is>
+      </c>
+      <c r="H76" s="26" t="inlineStr">
+        <is>
+          <t>Lupin FDA approval April 8, 2026. Lower-cost combination for T2D management.</t>
+        </is>
+      </c>
+      <c r="I76" s="26" t="inlineStr">
+        <is>
+          <t>FDA Approved (Generic)</t>
+        </is>
+      </c>
+      <c r="J76" s="26" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K76" s="26" t="inlineStr">
+        <is>
+          <t>https://www.prismnews.com/news/lupin-wins-fda-approval-for-generic-dapagliflozin-metformin</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="26" t="inlineStr">
+        <is>
+          <t>Cross</t>
+        </is>
+      </c>
+      <c r="B77" s="26" t="inlineStr">
+        <is>
+          <t>GLP-1 - Oral</t>
+        </is>
+      </c>
+      <c r="C77" s="26" t="inlineStr">
+        <is>
+          <t>Oral Semaglutide 25mg (Wegovy)</t>
+        </is>
+      </c>
+      <c r="D77" s="26" t="inlineStr">
+        <is>
+          <t>Novo Nordisk</t>
+        </is>
+      </c>
+      <c r="E77" s="26" t="inlineStr">
+        <is>
+          <t>Oral GLP-1 RA for weight loss</t>
+        </is>
+      </c>
+      <c r="F77" s="26" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="G77" s="26" t="inlineStr">
+        <is>
+          <t>First oral GLP-1 for weight management</t>
+        </is>
+      </c>
+      <c r="H77" s="26" t="inlineStr">
+        <is>
+          <t>FDA approved late 2025/early 2026. First GLP-1 pill for weight loss. Launched in US Jan 2026.</t>
+        </is>
+      </c>
+      <c r="I77" s="26" t="inlineStr">
+        <is>
+          <t>FDA Approved</t>
+        </is>
+      </c>
+      <c r="J77" s="26" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K77" s="26" t="inlineStr">
+        <is>
+          <t>https://www.ajmc.com/view/fda-approves-oral-semaglutide-as-first-glp-1-pill-for-weight-loss</t>
         </is>
       </c>
     </row>
@@ -5479,7 +5705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K40"/>
+  <dimension ref="A1:K44"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="35" customWidth="1" style="12" min="1" max="1"/>
@@ -7531,6 +7757,218 @@
       <c r="K40" s="12" t="inlineStr">
         <is>
           <t>https://doi.org/10.1186/s12911-026-03420-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="26" t="inlineStr">
+        <is>
+          <t>SGLT2i + Colchicine Combo in CAD+T2DM (TriNetX)</t>
+        </is>
+      </c>
+      <c r="B41" s="26" t="inlineStr">
+        <is>
+          <t>TriNetX Retrospective</t>
+        </is>
+      </c>
+      <c r="C41" s="26" t="inlineStr">
+        <is>
+          <t>TBD (PMID 40907678)</t>
+        </is>
+      </c>
+      <c r="D41" s="26" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E41" s="26" t="inlineStr">
+        <is>
+          <t>T2D/CV</t>
+        </is>
+      </c>
+      <c r="F41" s="26" t="inlineStr">
+        <is>
+          <t>Drug Combination</t>
+        </is>
+      </c>
+      <c r="G41" s="26" t="inlineStr">
+        <is>
+          <t>12,235 matched pts/arm; significant MACE, mortality, HF reduction vs colchicine alone. Retrospective only.</t>
+        </is>
+      </c>
+      <c r="H41" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="I41" s="26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J41" s="26" t="inlineStr">
+        <is>
+          <t>PARTIALLY_VALIDATED. No prospective RCT registered. Hypothesis-generating. Vetting date: 2026-04-13.</t>
+        </is>
+      </c>
+      <c r="K41" s="26" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/40907678/</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="26" t="inlineStr">
+        <is>
+          <t>Toward Personalized Medicine in T1D (Teplizumab)</t>
+        </is>
+      </c>
+      <c r="B42" s="26" t="inlineStr">
+        <is>
+          <t>Multiple</t>
+        </is>
+      </c>
+      <c r="C42" s="26" t="inlineStr">
+        <is>
+          <t>Diabetes Obes Metab</t>
+        </is>
+      </c>
+      <c r="D42" s="26" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E42" s="26" t="inlineStr">
+        <is>
+          <t>T1D</t>
+        </is>
+      </c>
+      <c r="F42" s="26" t="inlineStr">
+        <is>
+          <t>Immunotherapy / Personalized</t>
+        </is>
+      </c>
+      <c r="G42" s="26" t="inlineStr">
+        <is>
+          <t>Identifies exhausted T-cell phenotypes (PD-1+, TIGIT+, KLRG1+) predicting teplizumab response; recommends stage 2 intervention window.</t>
+        </is>
+      </c>
+      <c r="H42" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="I42" s="26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J42" s="26" t="inlineStr">
+        <is>
+          <t>HIGH relevance to teplizumab decision prep. Stratification biomarkers for patient selection.</t>
+        </is>
+      </c>
+      <c r="K42" s="26" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/41913320/</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="26" t="inlineStr">
+        <is>
+          <t>Predicted Meta-Omics for Microbiome Studies</t>
+        </is>
+      </c>
+      <c r="B43" s="26" t="inlineStr">
+        <is>
+          <t>Multiple</t>
+        </is>
+      </c>
+      <c r="C43" s="26" t="inlineStr">
+        <is>
+          <t>PLoS ONE</t>
+        </is>
+      </c>
+      <c r="D43" s="26" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E43" s="26" t="inlineStr">
+        <is>
+          <t>Cross</t>
+        </is>
+      </c>
+      <c r="F43" s="26" t="inlineStr">
+        <is>
+          <t>AI/ML + Microbiome</t>
+        </is>
+      </c>
+      <c r="G43" s="26" t="inlineStr">
+        <is>
+          <t>ML models predicting metabolite/transcript abundances from metagenomics; validated on IBD classification (r=0.74-0.77).</t>
+        </is>
+      </c>
+      <c r="H43" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="I43" s="26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J43" s="26" t="inlineStr">
+        <is>
+          <t>HIGH relevance to microbiome-ML pipeline research path. Cross-domain: AI/ML + Microbiome.</t>
+        </is>
+      </c>
+      <c r="K43" s="26" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/41961886/</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="26" t="inlineStr">
+        <is>
+          <t>Text Messaging GLP-1 Transition in Safety-Net Care</t>
+        </is>
+      </c>
+      <c r="B44" s="26" t="inlineStr">
+        <is>
+          <t>Multiple</t>
+        </is>
+      </c>
+      <c r="C44" s="26" t="inlineStr">
+        <is>
+          <t>JMIR Formative Research</t>
+        </is>
+      </c>
+      <c r="D44" s="26" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E44" s="26" t="inlineStr">
+        <is>
+          <t>T2D</t>
+        </is>
+      </c>
+      <c r="F44" s="26" t="inlineStr">
+        <is>
+          <t>Health Equity + GLP-1</t>
+        </is>
+      </c>
+      <c r="G44" s="26" t="inlineStr">
+        <is>
+          <t>Pilot SMS program for basal insulin→GLP-1 transition in multilingual safety-net clinics.</t>
+        </is>
+      </c>
+      <c r="H44" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="I44" s="26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J44" s="26" t="inlineStr">
+        <is>
+          <t>MEDIUM-HIGH relevance. Bridges health equity + novel therapies. Cross-domain paper.</t>
+        </is>
+      </c>
+      <c r="K44" s="26" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/41955563/</t>
         </is>
       </c>
     </row>

</xml_diff>